<commit_message>
June 23 2025 changes
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTI0063910_VerifyCounterpartiesDetailsAreMappedFromOpportunityToEngagementAfterConversion.xlsx
+++ b/TestData/LV_TMTI0063910_VerifyCounterpartiesDetailsAreMappedFromOpportunityToEngagementAfterConversion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F71F793-2FB5-480C-A725-47298F975FDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F279D62-03C6-46B3-BC39-CCCB7D235570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="708" windowWidth="23256" windowHeight="12456" tabRatio="548" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUsers" sheetId="2" r:id="rId1"/>
@@ -313,13 +313,13 @@
     <t>Internal</t>
   </si>
   <si>
-    <t>C:\Users\vijay.kumar\Downloads\</t>
-  </si>
-  <si>
     <t>BUS - Business Services</t>
   </si>
   <si>
     <t>Jennie Stewart</t>
+  </si>
+  <si>
+    <t>C:\Users\vkumar0427\Downloads\</t>
   </si>
 </sst>
 </file>
@@ -722,7 +722,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B2" t="s">
         <v>20</v>
@@ -936,7 +936,7 @@
         <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E2" t="s">
         <v>51</v>
@@ -1062,7 +1062,7 @@
         <v>79</v>
       </c>
       <c r="D2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E2" t="s">
         <v>83</v>

</xml_diff>

<commit_message>
June 24 2025 changes
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTI0063910_VerifyCounterpartiesDetailsAreMappedFromOpportunityToEngagementAfterConversion.xlsx
+++ b/TestData/LV_TMTI0063910_VerifyCounterpartiesDetailsAreMappedFromOpportunityToEngagementAfterConversion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F279D62-03C6-46B3-BC39-CCCB7D235570}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1727359-EFF5-489B-B10E-6C1A119D4717}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -319,7 +319,7 @@
     <t>Jennie Stewart</t>
   </si>
   <si>
-    <t>C:\Users\vkumar0427\Downloads\</t>
+    <t>C:\Users\vijay.kumar\Downloads\</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
WaiveRFO field Aug 8 2025
</commit_message>
<xml_diff>
--- a/TestData/LV_TMTI0063910_VerifyCounterpartiesDetailsAreMappedFromOpportunityToEngagementAfterConversion.xlsx
+++ b/TestData/LV_TMTI0063910_VerifyCounterpartiesDetailsAreMappedFromOpportunityToEngagementAfterConversion.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1727359-EFF5-489B-B10E-6C1A119D4717}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB1BFC0F-3DC2-4FF1-B751-3BD1B7551936}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="548" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="StandardUsers" sheetId="2" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="94">
   <si>
     <t>James Craven</t>
   </si>
@@ -320,6 +320,12 @@
   </si>
   <si>
     <t>C:\Users\vijay.kumar\Downloads\</t>
+  </si>
+  <si>
+    <t>MassEditComments</t>
+  </si>
+  <si>
+    <t>These are counterparty comments from Counterparty List page</t>
   </si>
 </sst>
 </file>
@@ -1024,7 +1030,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{751812A8-ABA8-4232-9D81-14F299F55479}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.28515625" bestFit="1" customWidth="1"/>
@@ -1032,9 +1038,10 @@
     <col min="3" max="3" width="42.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="57.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
@@ -1050,8 +1057,11 @@
       <c r="E1" s="1" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1067,8 +1077,11 @@
       <c r="E2" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>88</v>
       </c>

</xml_diff>